<commit_message>
Organize basic Excel projects
</commit_message>
<xml_diff>
--- a/FirstSheet.xlsx
+++ b/FirstSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8952172-AA94-463F-BAE5-7255A6707569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F56FBE0-D343-4A0B-AE32-749B73909BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1A666E1F-5257-43EE-9B24-0E1159324009}"/>
+    <workbookView minimized="1" xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{1A666E1F-5257-43EE-9B24-0E1159324009}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
   <si>
     <t>S.No</t>
   </si>
@@ -63,13 +63,73 @@
   </si>
   <si>
     <t>Madan Mohan</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weeks and Months </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,16 +137,72 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -94,12 +210,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,69 +588,569 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1E62C9C-1227-46FA-8870-468C93F746DF}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
+      <c r="E1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="4">
+        <v>1</v>
+      </c>
+      <c r="H1" s="4">
+        <v>11</v>
+      </c>
+      <c r="I1" s="4">
+        <v>21</v>
+      </c>
+      <c r="J1" s="4">
+        <v>31</v>
+      </c>
+      <c r="K1" s="4">
+        <v>41</v>
+      </c>
+      <c r="L1" s="4">
+        <v>51</v>
+      </c>
+      <c r="M1" s="4">
+        <v>61</v>
+      </c>
+      <c r="N1" s="4">
+        <v>71</v>
+      </c>
+      <c r="O1" s="4">
+        <v>81</v>
+      </c>
+      <c r="P1" s="4">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A2" s="1">
         <v>101</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>6397437304</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="6">
+        <v>2</v>
+      </c>
+      <c r="H2" s="5">
+        <v>2</v>
+      </c>
+      <c r="I2" s="5">
+        <v>2</v>
+      </c>
+      <c r="J2" s="5">
+        <v>2</v>
+      </c>
+      <c r="K2" s="5">
+        <v>2</v>
+      </c>
+      <c r="L2" s="5">
+        <v>2</v>
+      </c>
+      <c r="M2" s="5">
+        <v>2</v>
+      </c>
+      <c r="N2" s="5">
+        <v>2</v>
+      </c>
+      <c r="O2" s="5">
+        <v>82</v>
+      </c>
+      <c r="P2" s="5">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A3" s="1">
         <v>102</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>1546987562</v>
       </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="7">
+        <v>3</v>
+      </c>
+      <c r="H3" s="4">
+        <v>13</v>
+      </c>
+      <c r="I3" s="4">
+        <v>23</v>
+      </c>
+      <c r="J3" s="4">
+        <v>33</v>
+      </c>
+      <c r="K3" s="4">
+        <v>43</v>
+      </c>
+      <c r="L3" s="4">
+        <v>53</v>
+      </c>
+      <c r="M3" s="4">
+        <v>63</v>
+      </c>
+      <c r="N3" s="4">
+        <v>73</v>
+      </c>
+      <c r="O3" s="4">
+        <v>83</v>
+      </c>
+      <c r="P3" s="4">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A4" s="1">
         <v>103</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>5698741236</v>
       </c>
-      <c r="D4" t="s">
-        <v>5</v>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="6">
+        <v>4</v>
+      </c>
+      <c r="H4" s="5">
+        <v>14</v>
+      </c>
+      <c r="I4" s="5">
+        <v>24</v>
+      </c>
+      <c r="J4" s="5">
+        <v>34</v>
+      </c>
+      <c r="K4" s="5">
+        <v>44</v>
+      </c>
+      <c r="L4" s="5">
+        <v>54</v>
+      </c>
+      <c r="M4" s="5">
+        <v>64</v>
+      </c>
+      <c r="N4" s="5">
+        <v>74</v>
+      </c>
+      <c r="O4" s="5">
+        <v>84</v>
+      </c>
+      <c r="P4" s="5">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A5" s="1">
+        <v>104</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3849025966</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="7">
+        <v>5</v>
+      </c>
+      <c r="H5" s="4">
+        <v>15</v>
+      </c>
+      <c r="I5" s="4">
+        <v>25</v>
+      </c>
+      <c r="J5" s="4">
+        <v>35</v>
+      </c>
+      <c r="K5" s="4">
+        <v>45</v>
+      </c>
+      <c r="L5" s="4">
+        <v>55</v>
+      </c>
+      <c r="M5" s="4">
+        <v>65</v>
+      </c>
+      <c r="N5" s="4">
+        <v>75</v>
+      </c>
+      <c r="O5" s="4">
+        <v>85</v>
+      </c>
+      <c r="P5" s="4">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A6" s="1">
+        <v>105</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3499677932</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="6">
+        <v>6</v>
+      </c>
+      <c r="H6" s="5">
+        <v>16</v>
+      </c>
+      <c r="I6" s="5">
+        <v>26</v>
+      </c>
+      <c r="J6" s="5">
+        <v>36</v>
+      </c>
+      <c r="K6" s="5">
+        <v>46</v>
+      </c>
+      <c r="L6" s="5">
+        <v>56</v>
+      </c>
+      <c r="M6" s="5">
+        <v>66</v>
+      </c>
+      <c r="N6" s="5">
+        <v>76</v>
+      </c>
+      <c r="O6" s="5">
+        <v>86</v>
+      </c>
+      <c r="P6" s="5">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A7" s="1">
+        <v>106</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1">
+        <v>3150329898</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="7">
+        <v>7</v>
+      </c>
+      <c r="H7" s="4">
+        <v>17</v>
+      </c>
+      <c r="I7" s="4">
+        <v>27</v>
+      </c>
+      <c r="J7" s="4">
+        <v>37</v>
+      </c>
+      <c r="K7" s="4">
+        <v>47</v>
+      </c>
+      <c r="L7" s="4">
+        <v>57</v>
+      </c>
+      <c r="M7" s="4">
+        <v>67</v>
+      </c>
+      <c r="N7" s="4">
+        <v>77</v>
+      </c>
+      <c r="O7" s="4">
+        <v>87</v>
+      </c>
+      <c r="P7" s="4">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A8" s="1">
+        <v>107</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2800981864</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="6">
+        <v>8</v>
+      </c>
+      <c r="H8" s="5">
+        <v>18</v>
+      </c>
+      <c r="I8" s="5">
+        <v>28</v>
+      </c>
+      <c r="J8" s="5">
+        <v>38</v>
+      </c>
+      <c r="K8" s="5">
+        <v>48</v>
+      </c>
+      <c r="L8" s="5">
+        <v>58</v>
+      </c>
+      <c r="M8" s="5">
+        <v>68</v>
+      </c>
+      <c r="N8" s="5">
+        <v>78</v>
+      </c>
+      <c r="O8" s="5">
+        <v>88</v>
+      </c>
+      <c r="P8" s="5">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A9" s="1">
+        <v>108</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2451633830</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="7">
+        <v>9</v>
+      </c>
+      <c r="H9" s="4">
+        <v>19</v>
+      </c>
+      <c r="I9" s="4">
+        <v>29</v>
+      </c>
+      <c r="J9" s="4">
+        <v>39</v>
+      </c>
+      <c r="K9" s="4">
+        <v>49</v>
+      </c>
+      <c r="L9" s="4">
+        <v>59</v>
+      </c>
+      <c r="M9" s="4">
+        <v>69</v>
+      </c>
+      <c r="N9" s="4">
+        <v>79</v>
+      </c>
+      <c r="O9" s="4">
+        <v>89</v>
+      </c>
+      <c r="P9" s="4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A10" s="1">
+        <v>109</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1">
+        <v>2102285796</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="6">
+        <v>10</v>
+      </c>
+      <c r="H10" s="5">
+        <v>20</v>
+      </c>
+      <c r="I10" s="5">
+        <v>30</v>
+      </c>
+      <c r="J10" s="5">
+        <v>40</v>
+      </c>
+      <c r="K10" s="5">
+        <v>50</v>
+      </c>
+      <c r="L10" s="5">
+        <v>60</v>
+      </c>
+      <c r="M10" s="5">
+        <v>70</v>
+      </c>
+      <c r="N10" s="5">
+        <v>80</v>
+      </c>
+      <c r="O10" s="5">
+        <v>90</v>
+      </c>
+      <c r="P10" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A11" s="1">
+        <v>110</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1752937762</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A12" s="1">
+        <v>111</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1403589728</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.45">
+      <c r="A13" s="1">
+        <v>112</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1054241694</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:F1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>